<commit_message>
Implemented Olivia Text Draft
</commit_message>
<xml_diff>
--- a/Noir Wingman/Assets/Sheets/Olivia Meadows/OliviaDialogue 0.1.xlsx
+++ b/Noir Wingman/Assets/Sheets/Olivia Meadows/OliviaDialogue 0.1.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\coles\OneDrive\Desktop\NoirWingman\Noir Wingman\Assets\Sheets\Olivia Meadows\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{447B5ECF-5DF6-4088-A7F5-719C1931654B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{6EDECFC7-95E3-4C4E-A821-48A388CB1988}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15620" xr2:uid="{B7F00FD3-8E02-462F-86DF-9F799A3EC4EB}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="61">
   <si>
     <t>Name</t>
   </si>
@@ -95,9 +95,6 @@
     <t>What brings a nice reporter like you to a shithole like this, hm? Following a case?</t>
   </si>
   <si>
-    <t>For someone who loves asking hard questions, you don’t seem to enjoy being on the receiving end. Tell me more about why you ordered an egg cream.</t>
-  </si>
-  <si>
     <t>Elaborate on egg cream</t>
   </si>
   <si>
@@ -119,13 +116,112 @@
     <t>What kind of things do you report on? Puff pieces, human interest, politics, or-</t>
   </si>
   <si>
-    <t>Nah, long day- needed a drink somethin' fierce, and the egg creams here are second to none.</t>
-  </si>
-  <si>
-    <t>Sad</t>
-  </si>
-  <si>
     <t>Null</t>
+  </si>
+  <si>
+    <t>3|0</t>
+  </si>
+  <si>
+    <t>Olivia Meadows| Detective Juels</t>
+  </si>
+  <si>
+    <t>Nah, long day- needed a drink somethin' fierce, and the egg creams here are second to none.|You come to a Speakeasy- the Black Needle, no less- and you decide to order an egg cream? | Uh, yup! Booze slows me down, y'know?|*The gleam in her eye tells me there's more to that then she's telling me.|Are you sure that's it Ms.Meadows?|Who cares? Why are you even asking me this stuff!|*Hm. Maybe I can come back to this line of questioning later, once I know her more.</t>
+  </si>
+  <si>
+    <t>Sad|Neutral|Happy|Angry|Neutral|Angry|Angry</t>
+  </si>
+  <si>
+    <t>3|0|3|0|0|2|0</t>
+  </si>
+  <si>
+    <t>Like I said. I'm a reporter for the City Coronet|*Crap- She already said that!</t>
+  </si>
+  <si>
+    <t>Olivia Meadows|Detective Juels</t>
+  </si>
+  <si>
+    <t>Neutral|Sad</t>
+  </si>
+  <si>
+    <t>Sad|Sad|Sad|Neutral</t>
+  </si>
+  <si>
+    <t>2|2|3|0</t>
+  </si>
+  <si>
+    <t>Olivia Meadows|Olivia Meadows|Olivia Meadows|Detective Juels</t>
+  </si>
+  <si>
+    <t>My old man became an alcoholic after he got divorced from my mom-|*For the first time, her words slow to a comprehensible pace| I loved him- sad and drunk though he was- but I don't want to turn out like him. Happy?|Yeah, Peachy</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> No, no, I'm here alone. I'm actually new to the City.|Moved for the job, then?|University, actually, but it got me a job- you know that case on the Crab-Claw Cutter? |The one who kept murdering dock workers with- |With a crab claw, yup- I was the one who broke that story! The local rag hired me on the spot.</t>
+  </si>
+  <si>
+    <t>Neutral|Happy|Happy|Angry|Happy</t>
+  </si>
+  <si>
+    <t>3|0|3|0|2</t>
+  </si>
+  <si>
+    <t>Olivia Meadows|Detective Juels|Olivia Meadows|Detective Juels|Olivia Meadows</t>
+  </si>
+  <si>
+    <t>Why, you interested?|No, Not Particularly|Why Do you ask?|Plain Curiosity Ma'am|Oh, alright- yeah, no. I'm not opposed, I don't think, but I've been as busy as a bumblebee with my reporting.|Would you be open to going on a date with someone? |Well, I usually don't have time for that sorta thing. I dunno, guess it depends on who and what and where and why.</t>
+  </si>
+  <si>
+    <t>Neutral|Neutral|Neutral|Neutral|Neutral|Angry|Neutral</t>
+  </si>
+  <si>
+    <t>3|0|3|0|3|0|3</t>
+  </si>
+  <si>
+    <t>Olivia Meadows|Detective Juels|Olivia Meadows|Detective Juels|Olivia Meadows|Detective Juels|Olivia Meadows</t>
+  </si>
+  <si>
+    <t>Happy|Sad</t>
+  </si>
+  <si>
+    <t>Well, normally, I report on human interest stuff- puff pieces, y'know? But, what I'm really in this business for- what I care about, I guess- is corruption. Politicians, big corporations, you name it.| *Woah,  That certainly riled her up</t>
+  </si>
+  <si>
+    <t>1|0</t>
+  </si>
+  <si>
+    <t>The Fuzz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What do you think of the fuzz? </t>
+  </si>
+  <si>
+    <t>I meannn, come on. There's no institution more packed with corruption, bribery, bigotry, kickbacks, and blackmail than the fuzz. It's rotten, all the way to the core.|What about the people who work for them? |I mean, there are some folks who join for the right reasons, I guess- wanting to help people, protect their communities, all that- but still, a handful of termites- willing termites especially- can't clean up a mound made of manure.|You sound like you care a lot about this kind of thing.|I do, I really really do- it's all about asking the hard questions, y'know?| *Hypocrisy- she hates that. This might be my line!|Trust me, I do.</t>
+  </si>
+  <si>
+    <t>Angry|Neutral|Neutral|Happy|Happy|Angry|Neutral</t>
+  </si>
+  <si>
+    <t>3|0|3|0|3|0|0</t>
+  </si>
+  <si>
+    <t>Olivia Meadows|Detective Juels|Olivia Meadows|Detective Juels|Olivia Meadows|Detective Juels|Detective Juels</t>
+  </si>
+  <si>
+    <t>For someone who loves asking hard questions, you don't seem to enjoy being on the receiving end. Tell me more about why you ordered an egg cream.</t>
+  </si>
+  <si>
+    <t>Length</t>
+  </si>
+  <si>
+    <t>Add</t>
+  </si>
+  <si>
+    <t>Alcohol</t>
+  </si>
+  <si>
+    <t>egt</t>
+  </si>
+  <si>
+    <t>Olivia Meadows| Detective Juels|Olivia Meadows|Detective Juels|Detective Juels|Olivia Meadows|Detective Juels</t>
   </si>
 </sst>
 </file>
@@ -161,12 +257,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -501,13 +596,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B53663D6-615F-4D5D-A79A-E624F019796E}">
-  <dimension ref="A1:N7"/>
+  <dimension ref="A1:N8"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="19.90625" customWidth="1"/>
     <col min="2" max="2" width="43.36328125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="87.1796875" style="2" customWidth="1"/>
-    <col min="4" max="4" width="12" customWidth="1"/>
+    <col min="3" max="3" width="87.1796875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="13.54296875" style="1" customWidth="1"/>
+    <col min="5" max="5" width="14.08984375" customWidth="1"/>
+    <col min="6" max="6" width="14.1796875" customWidth="1"/>
+    <col min="7" max="7" width="15.7265625" customWidth="1"/>
+    <col min="9" max="9" width="10.1796875" customWidth="1"/>
+    <col min="10" max="10" width="11" customWidth="1"/>
+    <col min="11" max="11" width="14.453125" customWidth="1"/>
+    <col min="12" max="12" width="22" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.35">
@@ -517,7 +619,7 @@
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
@@ -561,158 +663,304 @@
       <c r="B2" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="C2" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>33</v>
+      </c>
       <c r="E2" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="F2" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="G2">
         <v>0</v>
       </c>
       <c r="H2" t="s">
-        <v>28</v>
+        <v>56</v>
       </c>
       <c r="I2" t="s">
-        <v>28</v>
+        <v>57</v>
       </c>
       <c r="J2">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="K2" t="s">
+        <v>26</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="M2">
+        <v>1</v>
+      </c>
+      <c r="N2">
+        <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:14" ht="29" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:14" ht="87" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>16</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="D3" t="s">
-        <v>27</v>
+      <c r="C3" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>29</v>
       </c>
       <c r="E3" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="F3" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="G3">
         <v>0</v>
       </c>
       <c r="H3" t="s">
-        <v>28</v>
+        <v>58</v>
       </c>
       <c r="I3" t="s">
-        <v>28</v>
+        <v>57</v>
       </c>
       <c r="J3">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="K3" t="s">
+        <v>30</v>
+      </c>
+      <c r="L3" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="M3">
+        <v>2</v>
+      </c>
+      <c r="N3">
+        <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:14" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="E4" t="s">
+        <v>58</v>
+      </c>
+      <c r="F4" t="s">
+        <v>59</v>
+      </c>
+      <c r="G4">
+        <v>1</v>
+      </c>
+      <c r="H4" t="s">
+        <v>56</v>
+      </c>
+      <c r="I4" t="s">
+        <v>57</v>
+      </c>
+      <c r="J4">
+        <v>1</v>
+      </c>
+      <c r="K4" t="s">
+        <v>35</v>
+      </c>
+      <c r="L4" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="M4">
+        <v>5</v>
+      </c>
+      <c r="N4">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" ht="87" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
         <v>19</v>
       </c>
-      <c r="B4" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="E4" t="s">
-        <v>28</v>
-      </c>
-      <c r="F4" t="s">
-        <v>28</v>
-      </c>
-      <c r="G4">
-        <v>0</v>
-      </c>
-      <c r="H4" t="s">
-        <v>28</v>
-      </c>
-      <c r="I4" t="s">
-        <v>28</v>
-      </c>
-      <c r="J4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
+      <c r="B5" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B5" s="1" t="s">
-        <v>21</v>
+      <c r="C5" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>39</v>
       </c>
       <c r="E5" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="F5" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="G5">
         <v>0</v>
       </c>
       <c r="H5" t="s">
-        <v>28</v>
+        <v>56</v>
       </c>
       <c r="I5" t="s">
-        <v>28</v>
+        <v>57</v>
       </c>
       <c r="J5">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="K5" t="s">
+        <v>40</v>
+      </c>
+      <c r="L5" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="M5">
+        <v>1</v>
+      </c>
+      <c r="N5">
+        <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:14" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
+        <v>21</v>
+      </c>
+      <c r="B6" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B6" s="1" t="s">
-        <v>23</v>
+      <c r="C6" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>43</v>
       </c>
       <c r="E6" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="F6" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="G6">
         <v>0</v>
       </c>
       <c r="H6" t="s">
-        <v>28</v>
+        <v>56</v>
       </c>
       <c r="I6" t="s">
-        <v>28</v>
+        <v>57</v>
       </c>
       <c r="J6">
+        <v>1</v>
+      </c>
+      <c r="K6" t="s">
+        <v>44</v>
+      </c>
+      <c r="L6" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="M6">
+        <v>2</v>
+      </c>
+      <c r="N6">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>23</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="E7" t="s">
+        <v>56</v>
+      </c>
+      <c r="F7" t="s">
+        <v>59</v>
+      </c>
+      <c r="G7">
+        <v>1</v>
+      </c>
+      <c r="H7" t="s">
+        <v>56</v>
+      </c>
+      <c r="I7" t="s">
+        <v>57</v>
+      </c>
+      <c r="J7">
+        <v>1</v>
+      </c>
+      <c r="K7" t="s">
+        <v>48</v>
+      </c>
+      <c r="L7" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="M7">
+        <v>-1</v>
+      </c>
+      <c r="N7">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" ht="101.5" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>49</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="G8">
+        <v>2</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="I8" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="J8">
+        <v>1</v>
+      </c>
+      <c r="K8" t="s">
+        <v>53</v>
+      </c>
+      <c r="L8" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="M8">
         <v>0</v>
       </c>
-    </row>
-    <row r="7" spans="1:14" ht="29" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
-        <v>24</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="E7" t="s">
-        <v>28</v>
-      </c>
-      <c r="F7" t="s">
-        <v>28</v>
-      </c>
-      <c r="G7">
-        <v>0</v>
-      </c>
-      <c r="H7" t="s">
-        <v>28</v>
-      </c>
-      <c r="I7" t="s">
-        <v>28</v>
-      </c>
-      <c r="J7">
+      <c r="N8">
         <v>0</v>
       </c>
     </row>

</xml_diff>